<commit_message>
application script - hanging output project customer
</commit_message>
<xml_diff>
--- a/1.training_model/model_config/application_results.xlsx
+++ b/1.training_model/model_config/application_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
           <t>REJECTION_REASON</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -492,7 +497,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>74.75</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -500,19 +505,20 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>98.7</v>
+        <v>99.39</v>
       </c>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HT275</t>
+          <t>LL510</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OILTEK</t>
+          <t>LIPICO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,26 +528,27 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SECTION 3</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>93.89</v>
-      </c>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>87.93000000000001</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>unseen CUSTOMER 'LIPICO'</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CPM6311</t>
+          <t>LL510</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -551,16 +558,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A1706</t>
+          <t>A1710</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SECTION 6</t>
+          <t>SECTION 1</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>84.31</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -568,245 +575,12 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>93.01000000000001</v>
+        <v>99.39</v>
       </c>
       <c r="H4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>FIT151</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>OILTEK</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SECTION 3</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>99.18000000000001</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>63.07</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>V29011</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>OILTEK</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>SECTION 3</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>62.48</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>97.37</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>PT500A</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>OILTEK</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SECTION 1</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>92.98</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>99.72</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ZZZ9999X</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>OILTEK</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>SECTION 6</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>77.90000000000001</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>93.01000000000001</v>
-      </c>
-      <c r="H8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LL510</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>UNKNOWN_CUSTOMER</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>unseen CUSTOMER 'UNKNOWN_CUSTOMER'</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>LL510</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>OILTEK</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>UNKNOWN_PROJECT</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>unseen PROJECT 'UNKNOWN_PROJECT'</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LL510</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>UNKNOWN_CUSTOMER</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>UNKNOWN_PROJECT</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>unseen CUSTOMER 'UNKNOWN_CUSTOMER'; unseen PROJECT 'UNKNOWN_PROJECT'</t>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>unseen PROJECT 'A1710' — prediction uses customer context only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refine prediction - application script
</commit_message>
<xml_diff>
--- a/1.training_model/model_config/application_results.xlsx
+++ b/1.training_model/model_config/application_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,7 +471,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>PROJECT_NOTE</t>
         </is>
       </c>
     </row>
@@ -518,32 +518,36 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LIPICO</t>
+          <t>OILTEK</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A1706</t>
+          <t>A1710</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>SECTION 2</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>96.83</v>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>unseen CUSTOMER 'LIPICO'</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>CLUSTER 1</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>99.62</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>unseen project 'A1710'</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -558,16 +562,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A1710</t>
+          <t>(not provided)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SECTION 1</t>
+          <t>SECTION 2</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>78.04000000000001</v>
+        <v>96.83</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -575,14 +579,49 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>99.39</v>
+        <v>99.62</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>unseen PROJECT 'A1710' — prediction uses customer context only</t>
-        </is>
-      </c>
+          <t>project not provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LL510</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LIPICO</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A1706</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>unseen CUSTOMER 'LIPICO' — please assign manually</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
training script - synthetic OOD injection
</commit_message>
<xml_diff>
--- a/1.training_model/model_config/application_results.xlsx
+++ b/1.training_model/model_config/application_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,37 +441,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>PROJECT</t>
+          <t>PREDICTED_SECTION</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>PREDICTED_SECTION</t>
+          <t>SECTION_CONFIDENCE</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>SECTION_CONFIDENCE</t>
+          <t>PREDICTED_CLUSTER</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>PREDICTED_CLUSTER</t>
+          <t>CLUSTER_CONFIDENCE</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>CLUSTER_CONFIDENCE</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>REJECTION_REASON</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>PROJECT_NOTE</t>
         </is>
       </c>
     </row>
@@ -488,32 +478,26 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
           <t>SECTION 1</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>78.04000000000001</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>57</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>CLUSTER 1</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>99.39</v>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>99.31</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LL510</t>
+          <t>LL001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -523,36 +507,26 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A1710</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>SECTION 2</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>96.83</v>
-      </c>
-      <c r="F3" t="inlineStr">
+          <t>SECTION 3</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>97.43000000000001</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>CLUSTER 1</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>99.62</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>unseen project 'A1710'</t>
-        </is>
-      </c>
+      <c r="F3" t="n">
+        <v>98.38</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LL510</t>
+          <t>LL0000000021</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -562,214 +536,108 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>(not provided)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>SECTION 2</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>96.83</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>99.62</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>project number is missing</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>numeric field width 10 digits exceeds training maximum of 6 digits — model was not trained on this format, prediction would be unreliable</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LL510</t>
+          <t>LL00000000102837</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LIPICO</t>
+          <t>OILTEK</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>unseen CUSTOMER 'LIPICO' — Please assign manually</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>numeric field width 14 digits exceeds training maximum of 6 digits — model was not trained on this format, prediction would be unreliable</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LL0000000021</t>
+          <t>LL510</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OILTEK</t>
+          <t>LIPICO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>SECTION 3</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>99.34999999999999</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>87.08</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>unseen CUSTOMER 'LIPICO' — Please assign manually</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LL0000000021</t>
+          <t>LL001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OILTEK</t>
+          <t>UNKNOWN_CO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A1710</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SECTION 3</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>98.89</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>92.2</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>unseen project 'A1710'</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>LL0000000021</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>OILTEK</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>(not provided)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>SECTION 3</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>98.89</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>CLUSTER 1</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>92.2</v>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>project number is missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LL0000000021</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>LIPICO</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>A1706</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>unseen CUSTOMER 'LIPICO' — Please assign manually</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>unseen CUSTOMER 'UNKNOWN_CO' — Please assign manually</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
application script - OOD, KNN, XGB
</commit_message>
<xml_diff>
--- a/1.training_model/model_config/application_results.xlsx
+++ b/1.training_model/model_config/application_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,11 +464,16 @@
           <t>REJECTION_REASON</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>FORMAT_WARNING</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LL510</t>
+          <t>LL001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -478,26 +483,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SECTION 1</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CLUSTER 1</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>99.31</v>
+        <v>5</v>
       </c>
       <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LL001</t>
+          <t>LL510</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -507,11 +513,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SECTION 3</t>
+          <t>SECTION 1</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>97.43000000000001</v>
+        <v>56.34</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -519,9 +525,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>98.38</v>
+        <v>98.08</v>
       </c>
       <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -539,16 +546,21 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>numeric field width 10 digits exceeds training maximum of 6 digits — model was not trained on this format, prediction would be unreliable</t>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>unusual format — numeric field width 10 digits exceeds training maximum of 6 digits (confidence penalised by KNN scorer)</t>
         </is>
       </c>
     </row>
@@ -568,16 +580,21 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>numeric field width 14 digits exceeds training maximum of 6 digits — model was not trained on this format, prediction would be unreliable</t>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>unusual format — numeric field width 14 digits exceeds training maximum of 6 digits (confidence penalised by KNN scorer)</t>
         </is>
       </c>
     </row>
@@ -609,6 +626,7 @@
           <t>unseen CUSTOMER 'LIPICO' — Please assign manually</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -638,6 +656,7 @@
           <t>unseen CUSTOMER 'UNKNOWN_CO' — Please assign manually</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
training,application - removal rank
</commit_message>
<xml_diff>
--- a/1.training_model/model_config/application_results.xlsx
+++ b/1.training_model/model_config/application_results.xlsx
@@ -513,11 +513,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SECTION 1</t>
+          <t>SECTION 2</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>56.34</v>
+        <v>92.70999999999999</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>98.08</v>
+        <v>98.05</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>

</xml_diff>

<commit_message>
redefine formula of prediction - application script
</commit_message>
<xml_diff>
--- a/1.training_model/model_config/application_results.xlsx
+++ b/1.training_model/model_config/application_results.xlsx
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>5.17</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>5.18</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>92.70999999999999</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>98.05</v>
+        <v>96.84</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>0.11</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>0.11</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>0.13</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>0.14</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">

</xml_diff>